<commit_message>
feat(F-NAR-019): TREE-COL-006 polish Le rayon du vestiaire de Mila
</commit_message>
<xml_diff>
--- a/stories/arbres/TREE-COL-006.xlsx
+++ b/stories/arbres/TREE-COL-006.xlsx
@@ -10110,17 +10110,17 @@
       </c>
       <c r="E49" s="2" t="inlineStr">
         <is>
-          <t>Le rayon du vestiaire traverse le coussin, puis s'en va. La virgule a failli s'étouffer, sous le bleu. Elle chante, sur nos genoux. Deux chansons, un bois nu. Nina tapote, plus léger. Papa plie l'écharpe, le fil d'or au bord. Maman a plié l'écharpe, le fil d'or caché.</t>
+          <t>Le rayon du vestiaire traverse le coussin, puis s'en va. La virgule a failli s'étouffer, sous le bleu. Elle chante, sur nos genoux. Deux chansons, un bois nu. Nina tapote, plus léger. Papa raccroche le ciré, au crochet voisin. Maman a plié l'écharpe, le fil d'or caché.</t>
         </is>
       </c>
       <c r="F49" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le rayon du vestiaire traverse le coussin, puis s'en va. La virgule a failli s'étouffer, sous le bleu. Elle chante, sur nos genoux. Deux chansons, un bois nu. Nina tapote, plus léger. Papa plie l'écharpe, le fil d'or au bord. Maman a plié l'écharpe, le fil d'or caché.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="slow" pitch="-2st"&gt;Le rayon du vestiaire traverse le coussin, puis s'en va. La virgule a failli s'étouffer, sous le bleu. Elle chante, sur nos genoux. Deux chansons, un bois nu. Nina tapote, plus léger. Papa raccroche le ciré, au crochet voisin. Maman a plié l'écharpe, le fil d'or caché.&lt;/prosody&gt;&lt;break time="900ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G49" s="2" t="inlineStr">
         <is>
-          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le rayon du vestiaire traverse le coussin, puis s'en va. La virgule a failli s'étouffer, sous le bleu. Elle chante, sur nos genoux. Deux chansons, un bois nu. Nina tapote, plus léger. Papa plie l'écharpe, le fil d'or au bord. Maman a plié l'écharpe, le fil d'or caché.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
+          <t>&lt;low-pitch&gt;&lt;soft&gt;&lt;slow&gt;Le rayon du vestiaire traverse le coussin, puis s'en va. La virgule a failli s'étouffer, sous le bleu. Elle chante, sur nos genoux. Deux chansons, un bois nu. Nina tapote, plus léger. Papa raccroche le ciré, au crochet voisin. Maman a plié l'écharpe, le fil d'or caché.&lt;/slow&gt;&lt;/soft&gt;&lt;/low-pitch&gt; [long-pause]</t>
         </is>
       </c>
       <c r="H49" s="2" t="inlineStr"/>
@@ -10263,7 +10263,7 @@
 enfant-f|Elle chante, sur nos genoux.
 maman|Deux chansons, un bois nu.
 narrateur|Nina tapote, plus léger.
-narrateur|Papa plie l'écharpe, le fil d'or au bord.
+narrateur|Papa raccroche le ciré, au crochet voisin.
 narrateur|Maman a plié l'écharpe, le fil d'or caché.</t>
         </is>
       </c>
@@ -13326,17 +13326,17 @@
       </c>
       <c r="E66" s="2" t="inlineStr">
         <is>
-          <t>Près de la fenêtre, Mila veut tracer l'or sur le verre. La virgule, sur la vitre ! Le ciel, sur la vitre ! Le crayon glisse, et un trait rate le ciel. Nina grogne, tout bas. Mila retire la mine, sans frotter. Dans le miroir, la vraie virgule d'or tient. Toi le ciel, dans l'eau. Toi l'or, sur le papier, pas sur le verre. La vitre a gardé un trait pâle, souvenir. Le livre a retrouvé le loup, au sec. Mila dessine l'or sur une feuille, loin du froid. Nina dit le ciel, en regardant la flaque. Le nuage de l'eau a cessé de trembler.</t>
+          <t>Près de la fenêtre, Mila veut tracer l'or sur le verre. La virgule, sur la vitre ! Le ciel, sur la vitre ! Le crayon glisse, et un trait rate le ciel. Nina souffle, tout bas. Mila retire la mine, sans frotter. Dans le miroir, la vraie virgule d'or tient. Toi le ciel, dans l'eau. Toi l'or, sur le papier, pas sur le verre. La vitre a gardé un trait pâle, souvenir. Le livre a retrouvé le loup, au sec. Mila dessine l'or sur une feuille, loin du froid. Nina dit le ciel, en regardant la flaque. Le nuage de l'eau a cessé de trembler.</t>
         </is>
       </c>
       <c r="F66" s="2" t="inlineStr">
         <is>
-          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Près de la fenêtre, Mila veut tracer l'or sur le verre. La virgule, sur la vitre ! Le ciel, sur la vitre ! Le crayon glisse, et un trait rate le ciel. Nina grogne, tout bas. Mila retire la mine, sans frotter. Dans le miroir, la vraie &lt;emphasis level="moderate"&gt;virgule d'or&lt;/emphasis&gt; tient. Toi le ciel, dans l'eau. Toi l'or, sur le papier, pas sur le verre. La vitre a gardé un trait pâle, souvenir. Le livre a retrouvé le loup, au sec. Mila dessine l'or sur une feuille, loin du froid. Nina dit le ciel, en regardant la flaque. Le nuage de l'eau a cessé de trembler.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
+          <t>&lt;speak&gt;&lt;prosody rate="medium" pitch="medium"&gt;Près de la fenêtre, Mila veut tracer l'or sur le verre. La virgule, sur la vitre ! Le ciel, sur la vitre ! Le crayon glisse, et un trait rate le ciel. Nina souffle, tout bas. Mila retire la mine, sans frotter. Dans le miroir, la vraie &lt;emphasis level="moderate"&gt;virgule d'or&lt;/emphasis&gt; tient. Toi le ciel, dans l'eau. Toi l'or, sur le papier, pas sur le verre. La vitre a gardé un trait pâle, souvenir. Le livre a retrouvé le loup, au sec. Mila dessine l'or sur une feuille, loin du froid. Nina dit le ciel, en regardant la flaque. Le nuage de l'eau a cessé de trembler.&lt;/prosody&gt;&lt;break time="560ms"/&gt;&lt;/speak&gt;</t>
         </is>
       </c>
       <c r="G66" s="2" t="inlineStr">
         <is>
-          <t>Près de la fenêtre, Mila veut tracer l'or sur le verre. La virgule, sur la vitre ! Le ciel, sur la vitre ! Le crayon glisse, et un trait rate le ciel. Nina grogne, tout bas. Mila retire la mine, sans frotter. Dans le miroir, la vraie &lt;emphasis&gt;virgule d'or&lt;/emphasis&gt; tient. Toi le ciel, dans l'eau. Toi l'or, sur le papier, pas sur le verre. La vitre a gardé un trait pâle, souvenir. Le livre a retrouvé le loup, au sec. Mila dessine l'or sur une feuille, loin du froid. Nina dit le ciel, en regardant la flaque. Le nuage de l'eau a cessé de trembler. [pause]</t>
+          <t>Près de la fenêtre, Mila veut tracer l'or sur le verre. La virgule, sur la vitre ! Le ciel, sur la vitre ! Le crayon glisse, et un trait rate le ciel. Nina souffle, tout bas. Mila retire la mine, sans frotter. Dans le miroir, la vraie &lt;emphasis&gt;virgule d'or&lt;/emphasis&gt; tient. Toi le ciel, dans l'eau. Toi l'or, sur le papier, pas sur le verre. La vitre a gardé un trait pâle, souvenir. Le livre a retrouvé le loup, au sec. Mila dessine l'or sur une feuille, loin du froid. Nina dit le ciel, en regardant la flaque. Le nuage de l'eau a cessé de trembler. [pause]</t>
         </is>
       </c>
       <c r="H66" s="2" t="inlineStr"/>
@@ -13474,7 +13474,7 @@
 enfant-f|La virgule, sur la vitre !
 copine|Le ciel, sur la vitre !
 narrateur|Le crayon glisse, et un trait rate le ciel.
-narrateur|Nina grogne, tout bas.
+narrateur|Nina souffle, tout bas.
 narrateur|Mila retire la mine, sans frotter.
 narrateur|Dans le miroir, la vraie virgule d'or tient.
 enfant-f|Toi le ciel, dans l'eau.
@@ -17477,7 +17477,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:A18"/>
+  <dimension ref="A1:A19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="100" customWidth="1" min="1" max="1"/>
@@ -17604,6 +17604,13 @@
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
+        <is>
+          <t>F-NAR-008 récit, pas une leçon en puces</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" t="inlineStr">
         <is>
           <t>F-NAR-008 récit, pas une leçon en puces</t>
         </is>

</xml_diff>